<commit_message>
docs(plan): mark Nhanh sprint 3 backend tasks ready for review
SePay reconciliation, expiry job, refunds, claims and SePay sync are done on
sprint-3/be-nhanh; screens for these tasks stay with Khai and Khoi.
</commit_message>
<xml_diff>
--- a/docs/ke-hoach/SWP391_TaskSheet_Sprint3.xlsx
+++ b/docs/ke-hoach/SWP391_TaskSheet_Sprint3.xlsx
@@ -1717,12 +1717,12 @@
       </c>
       <c r="K21" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L21" s="23" t="inlineStr">
         <is>
-          <t>Hiện chỉ đánh dấu hết hạn khi hội viên tạo hoá đơn mới (expireStalePendingInvoices); chưa có job nền</t>
+          <t>BE xong 14/10/2026 trên sprint-3/be-nhanh, 143 test BE pass; chờ review/merge</t>
         </is>
       </c>
     </row>
@@ -1779,12 +1779,12 @@
       </c>
       <c r="K22" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L22" s="23" t="inlineStr">
         <is>
-          <t>Giao dịch lệch đã lưu ở payment_webhook_logs; chưa có API và màn xử lý</t>
+          <t>BE xong 14/10/2026 trên sprint-3/be-nhanh, 143 test BE pass; chờ review/merge</t>
         </is>
       </c>
     </row>
@@ -1903,12 +1903,12 @@
       </c>
       <c r="K24" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L24" s="23" t="inlineStr">
         <is>
-          <t>Đã có danh sách hoá đơn lọc theo kênh, chi tiết và biên lai; chưa có bảng thanh toán (payments)</t>
+          <t>BE xong 14/10/2026 trên sprint-3/be-nhanh, 143 test BE pass; chờ review/merge</t>
         </is>
       </c>
     </row>
@@ -2027,12 +2027,12 @@
       </c>
       <c r="K26" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L26" s="23" t="inlineStr">
         <is>
-          <t>Cần nhóm chốt: hoàn toàn bộ thì trừ lại số ngày đã cộng vào membership; hoàn phần thừa thì không đổi gói (#90).</t>
+          <t>BE xong 14/10/2026 trên sprint-3/be-nhanh, 143 test BE pass; chờ review/merge</t>
         </is>
       </c>
     </row>
@@ -3879,10 +3879,14 @@
       </c>
       <c r="K56" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="L56" s="23" t="n"/>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="L56" s="23" t="inlineStr">
+        <is>
+          <t>BE xong 14/10/2026 trên sprint-3/be-nhanh, 143 test BE pass; chờ review/merge</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="87" customHeight="1" s="18">
       <c r="A57" s="22" t="inlineStr">
@@ -3995,10 +3999,14 @@
       </c>
       <c r="K58" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="L58" s="23" t="n"/>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="L58" s="23" t="inlineStr">
+        <is>
+          <t>BE xong 14/10/2026 trên sprint-3/be-nhanh, 143 test BE pass; chờ review/merge</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="73.5" customHeight="1" s="18">
       <c r="A59" s="22" t="inlineStr">
@@ -4111,10 +4119,14 @@
       </c>
       <c r="K60" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="L60" s="23" t="n"/>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="L60" s="23" t="inlineStr">
+        <is>
+          <t>BE xong 14/10/2026 trên sprint-3/be-nhanh, 143 test BE pass; chờ review/merge</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="73.5" customHeight="1" s="18">
       <c r="A61" s="22" t="inlineStr">
@@ -4227,10 +4239,14 @@
       </c>
       <c r="K62" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="L62" s="23" t="n"/>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="L62" s="23" t="inlineStr">
+        <is>
+          <t>BE xong 14/10/2026 trên sprint-3/be-nhanh, 143 test BE pass; chờ review/merge</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="87" customHeight="1" s="18">
       <c r="A63" s="22" t="inlineStr">
@@ -4343,10 +4359,14 @@
       </c>
       <c r="K64" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="L64" s="23" t="n"/>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="L64" s="23" t="inlineStr">
+        <is>
+          <t>BE xong 14/10/2026 trên sprint-3/be-nhanh, 143 test BE pass; chờ review/merge</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="73.5" customHeight="1" s="18">
       <c r="A65" s="22" t="inlineStr">
@@ -4459,10 +4479,14 @@
       </c>
       <c r="K66" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="L66" s="23" t="n"/>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="L66" s="23" t="inlineStr">
+        <is>
+          <t>BE xong 14/10/2026 trên sprint-3/be-nhanh, 143 test BE pass; chờ review/merge</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="87" customHeight="1" s="18">
       <c r="A67" s="22" t="inlineStr">
@@ -4575,10 +4599,14 @@
       </c>
       <c r="K68" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="L68" s="23" t="n"/>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="L68" s="23" t="inlineStr">
+        <is>
+          <t>BE xong 14/10/2026 trên sprint-3/be-nhanh, 143 test BE pass; chờ review/merge</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="87" customHeight="1" s="18">
       <c r="A69" s="22" t="inlineStr">
@@ -4633,10 +4661,14 @@
       </c>
       <c r="K69" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="L69" s="23" t="n"/>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="L69" s="23" t="inlineStr">
+        <is>
+          <t>BE xong 14/10/2026 trên sprint-3/be-nhanh, 143 test BE pass; chờ review/merge #95: BE đã cho hội viên tải biên lai của chính mình (GET /invoices/:id/receipt, quyền invoice.read_own), FE chỉ cần mở nút.</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="87" customHeight="1" s="18">
       <c r="A70" s="22" t="inlineStr">
@@ -4749,10 +4781,14 @@
       </c>
       <c r="K71" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="L71" s="23" t="n"/>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="L71" s="23" t="inlineStr">
+        <is>
+          <t>BE xong 14/10/2026 trên sprint-3/be-nhanh, 143 test BE pass; chờ review/merge</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="73.5" customHeight="1" s="18">
       <c r="A72" s="22" t="inlineStr">
@@ -5337,10 +5373,14 @@
       </c>
       <c r="K81" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="L81" s="23" t="n"/>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="L81" s="23" t="inlineStr">
+        <is>
+          <t>BE xong 14/10/2026 trên sprint-3/be-nhanh, 143 test BE pass; chờ review/merge</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="73.5" customHeight="1" s="18">
       <c r="A82" s="22" t="inlineStr">
@@ -7943,7 +7983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6171875" defaultRowHeight="13.5" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="8"/>
@@ -7956,7 +7996,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="13.5" customHeight="1" s="18">
       <c r="A3" s="26" t="inlineStr">
         <is>
@@ -8174,7 +8213,6 @@
         <v/>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="13.5" customHeight="1" s="18">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -8225,24 +8263,12 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>7. Manager xem nhật ký thao tác, dashboard báo cáo và xuất tệp</t>
         </is>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
feat(sprint3): implement Bao backend membership and class workflows
</commit_message>
<xml_diff>
--- a/docs/ke-hoach/SWP391_TaskSheet_Sprint3.xlsx
+++ b/docs/ke-hoach/SWP391_TaskSheet_Sprint3.xlsx
@@ -1105,7 +1105,7 @@
       </c>
       <c r="K11" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L11" s="23" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="K14" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L14" s="23" t="n"/>
@@ -1411,7 +1411,7 @@
       </c>
       <c r="K16" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L16" s="23" t="n"/>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="K28" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L28" s="23" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="K30" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L30" s="23" t="n"/>
@@ -3507,7 +3507,7 @@
       </c>
       <c r="K50" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L50" s="23" t="inlineStr">
@@ -3631,7 +3631,7 @@
       </c>
       <c r="K52" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L52" s="23" t="inlineStr">
@@ -5141,7 +5141,7 @@
       </c>
       <c r="K77" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L77" s="23" t="n"/>
@@ -5257,7 +5257,7 @@
       </c>
       <c r="K79" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L79" s="23" t="n"/>
@@ -5435,7 +5435,7 @@
       </c>
       <c r="K82" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L82" s="23" t="n"/>
@@ -5671,7 +5671,7 @@
       </c>
       <c r="K86" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L86" s="23" t="n"/>
@@ -5787,7 +5787,7 @@
       </c>
       <c r="K88" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L88" s="23" t="n"/>
@@ -5903,7 +5903,7 @@
       </c>
       <c r="K90" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L90" s="23" t="n"/>

</xml_diff>

<commit_message>
docs(sprint3): deliver Khoi task status and acceptance evidence
</commit_message>
<xml_diff>
--- a/docs/ke-hoach/SWP391_TaskSheet_Sprint3.xlsx
+++ b/docs/ke-hoach/SWP391_TaskSheet_Sprint3.xlsx
@@ -1349,7 +1349,7 @@
       </c>
       <c r="K15" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L15" s="23" t="inlineStr">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="K17" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L17" s="23" t="inlineStr">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="K27" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L27" s="23" t="inlineStr">
@@ -2213,7 +2213,7 @@
       </c>
       <c r="K29" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L29" s="23" t="inlineStr">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="K31" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L31" s="23" t="n"/>
@@ -3693,7 +3693,7 @@
       </c>
       <c r="K53" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L53" s="23" t="inlineStr">
@@ -3755,7 +3755,7 @@
       </c>
       <c r="K54" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L54" s="23" t="inlineStr">
@@ -3817,7 +3817,7 @@
       </c>
       <c r="K55" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L55" s="23" t="inlineStr">
@@ -4061,7 +4061,7 @@
       </c>
       <c r="K59" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L59" s="23" t="n"/>
@@ -4541,7 +4541,7 @@
       </c>
       <c r="K67" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L67" s="23" t="n"/>
@@ -4843,7 +4843,7 @@
       </c>
       <c r="K72" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L72" s="23" t="n"/>
@@ -4901,7 +4901,7 @@
       </c>
       <c r="K73" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L73" s="23" t="inlineStr">
@@ -4963,7 +4963,7 @@
       </c>
       <c r="K74" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L74" s="23" t="n"/>
@@ -5199,7 +5199,7 @@
       </c>
       <c r="K78" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L78" s="23" t="n"/>
@@ -5729,7 +5729,7 @@
       </c>
       <c r="K87" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L87" s="23" t="n"/>
@@ -5845,7 +5845,7 @@
       </c>
       <c r="K89" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L89" s="23" t="n"/>
@@ -6139,7 +6139,7 @@
       </c>
       <c r="K94" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L94" s="23" t="inlineStr">
@@ -6201,7 +6201,7 @@
       </c>
       <c r="K95" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L95" s="23" t="inlineStr">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="K96" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L96" s="23" t="inlineStr">
@@ -6821,7 +6821,7 @@
       </c>
       <c r="K105" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L105" s="23" t="inlineStr">
@@ -6883,7 +6883,7 @@
       </c>
       <c r="K106" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L106" s="23" t="inlineStr">
@@ -6945,7 +6945,7 @@
       </c>
       <c r="K107" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L107" s="23" t="inlineStr">
@@ -7131,7 +7131,7 @@
       </c>
       <c r="K110" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L110" s="23" t="inlineStr">
@@ -7193,7 +7193,7 @@
       </c>
       <c r="K111" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L111" s="23" t="inlineStr">
@@ -7317,7 +7317,7 @@
       </c>
       <c r="K113" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L113" s="23" t="inlineStr">
@@ -7627,7 +7627,7 @@
       </c>
       <c r="K118" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L118" s="23" t="inlineStr">
@@ -7689,7 +7689,7 @@
       </c>
       <c r="K119" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L119" s="23" t="inlineStr">
@@ -7751,7 +7751,7 @@
       </c>
       <c r="K120" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L120" s="23" t="inlineStr">
@@ -7875,7 +7875,7 @@
       </c>
       <c r="K122" s="22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L122" s="23" t="inlineStr">

</xml_diff>